<commit_message>
feat(surveys): DS-D# dimension IDs, v2 crosswalk in insights, v1 band statement
Developer Survey dimensions are DS-D2 to DS-D8 in outputs and in the
Learning Survey bank so they no longer collide with v2 D1 to D9; old Forms
text still parses. The insights link each DS dimension to the v2 questions
it helps validate.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
Copilot-Session: f9fd4a8a-033c-4218-b2f1-2c8da428242c
</commit_message>
<xml_diff>
--- a/survey-learning/template-export-forms-learning.xlsx
+++ b/survey-learning/template-export-forms-learning.xlsx
@@ -526,37 +526,37 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>L2-Q1: **D2 — Copilot Adoption** (modos Ask/Edit/Agent/Coding Agent, features, ganho mensurado): qual seu nível?</t>
+          <t>L2-Q1: **DS-D2 Copilot Adoption** (modos Ask/Edit/Agent/Coding Agent, features, ganho mensurado): qual seu nível?</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>L2-Q2: **D3 — Microsoft/GitHub Tooling** (Foundry, Spaces, Coding Agent, MCP, Spec Kit, GHAS): qual seu nível?</t>
+          <t>L2-Q2: **DS-D3 Microsoft/GitHub Tooling** (Foundry, Spaces, Coding Agent, MCP, Spec Kit, GHAS): qual seu nível?</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>L2-Q3: **D4 — AI Dev Practices** (TDD com IA, SDD, pair programming, debugging com IA): qual seu nível?</t>
+          <t>L2-Q3: **DS-D4 AI Dev Practices** (TDD com IA, SDD, pair programming, debugging com IA): qual seu nível?</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">L2-Q4: **D5 — Agent Concepts** (custom agents, skills, prompts, MCP, A2A, handoffs, subagentes, personas Agentic DevOps): qual </t>
+          <t xml:space="preserve">L2-Q4: **DS-D5 Agent Concepts** (custom agents, skills, prompts, MCP, A2A, handoffs, subagentes, personas Agentic DevOps): qual </t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>L2-Q5: **D6 — Instructions / Memory** (copilot-instructions.md, AGENTS.md, CLAUDE.md, Spaces, prompt library): qual seu nível?</t>
+          <t>L2-Q5: **DS-D6 Instructions / Memory** (copilot-instructions.md, AGENTS.md, CLAUDE.md, Spaces, prompt library): qual seu nível?</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>L2-Q6: **D7 — Best Practices** (Champion, métricas DORA/DX, comunidade, compartilha prompts): qual seu nível?</t>
+          <t>L2-Q6: **DS-D7 Best Practices** (Champion, métricas DORA/DX, comunidade, compartilha prompts): qual seu nível?</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>L2-Q7: **D8 — Security &amp; Governance** (política IA, GHAS, SBOM, JIT permissions, red-lines de agents, audit): qual seu nível?</t>
+          <t>L2-Q7: **DS-D8 Security &amp; Governance** (política IA, GHAS, SBOM, JIT permissions, red-lines de agents, audit): qual seu nível?</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>D8 — Security &amp; Governance (GHAS, SBOM, red-lines); D5 — Agent Concepts (custom agents, MCP, A2A)</t>
+          <t>DS-D8 Security &amp; Governance (GHAS, SBOM, red-lines); DS-D5 Agent Concepts (custom agents, MCP, A2A)</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -931,7 +931,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>D3 — MS/GitHub Tooling (Foundry, Spaces, Spec Kit, MCP); D6 — Instructions / Memory (instructions files, prompt library); D7 — Best Practices (DORA, comunidade, mentoria); D4 — AI Dev Practices (TDD com IA, SDD); D2 — Copilot Adoption (modos avançados, Coding Agent)</t>
+          <t>DS-D3 MS/GitHub Tooling (Foundry, Spaces, Spec Kit, MCP); DS-D6 Instructions / Memory (instructions files, prompt library); DS-D7 Best Practices (DORA, comunidade, mentoria); DS-D4 AI Dev Practices (TDD com IA, SDD); DS-D2 Copilot Adoption (modos avançados, Coding Agent)</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>D8 — Security &amp; Governance (GHAS, SBOM, red-lines); D5 — Agent Concepts (custom agents, MCP, A2A); D2 — Copilot Adoption (modos avançados, Coding Agent); D6 — Instructions / Memory (instructions files, prompt library); D7 — Best Practices (DORA, comunidade, mentoria)</t>
+          <t>DS-D8 Security &amp; Governance (GHAS, SBOM, red-lines); DS-D5 Agent Concepts (custom agents, MCP, A2A); DS-D2 Copilot Adoption (modos avançados, Coding Agent); DS-D6 Instructions / Memory (instructions files, prompt library); DS-D7 Best Practices (DORA, comunidade, mentoria)</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>D7 — Best Practices (DORA, comunidade, mentoria); D3 — MS/GitHub Tooling (Foundry, Spaces, Spec Kit, MCP); D2 — Copilot Adoption (modos avançados, Coding Agent); D6 — Instructions / Memory (instructions files, prompt library)</t>
+          <t>DS-D7 Best Practices (DORA, comunidade, mentoria); DS-D3 MS/GitHub Tooling (Foundry, Spaces, Spec Kit, MCP); DS-D2 Copilot Adoption (modos avançados, Coding Agent); DS-D6 Instructions / Memory (instructions files, prompt library)</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -1486,7 +1486,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>D3 — MS/GitHub Tooling (Foundry, Spaces, Spec Kit, MCP); D6 — Instructions / Memory (instructions files, prompt library)</t>
+          <t>DS-D3 MS/GitHub Tooling (Foundry, Spaces, Spec Kit, MCP); DS-D6 Instructions / Memory (instructions files, prompt library)</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -1614,9 +1614,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1631,9 +1629,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1648,9 +1644,7 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
+    <row r="8"/>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
@@ -1693,9 +1687,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr"/>
-    </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>

</xml_diff>